<commit_message>
Fix fraccionamientos documento de entrada
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica_subdivision.xlsx
+++ b/storage/app/public/ficha_tecnica_subdivision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ODS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8C3CE4-B3C7-4B56-9AE2-8FA5416E10F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9AE9DE-731B-41B3-BF86-730F103AB9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59A6636E-DD9B-4BB2-A6F8-8B43A0BBD60A}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="167">
   <si>
     <t>Cuenta Predial</t>
   </si>
@@ -527,6 +527,18 @@
   </si>
   <si>
     <t>descripcion</t>
+  </si>
+  <si>
+    <t>GRAVAMEN</t>
+  </si>
+  <si>
+    <t>ACTO</t>
+  </si>
+  <si>
+    <t>acto contenido</t>
+  </si>
+  <si>
+    <t>descripcion acto</t>
   </si>
 </sst>
 </file>
@@ -630,7 +642,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -656,6 +668,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -971,7 +986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CE6CF71-2ADA-45B0-88E2-9CF8220A3B5B}">
-  <dimension ref="A1:BC14"/>
+  <dimension ref="A1:BE14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -1025,9 +1040,11 @@
     <col min="53" max="53" width="35.85546875" customWidth="1"/>
     <col min="54" max="54" width="36.28515625" customWidth="1"/>
     <col min="55" max="55" width="44.28515625" customWidth="1"/>
+    <col min="56" max="56" width="35.42578125" customWidth="1"/>
+    <col min="57" max="57" width="43.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:55" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:57" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1085,7 +1102,9 @@
       <c r="AU1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AV1" s="9"/>
+      <c r="AV1" s="9" t="s">
+        <v>163</v>
+      </c>
       <c r="AW1" s="9"/>
       <c r="AX1" s="9"/>
       <c r="AY1" s="9"/>
@@ -1093,8 +1112,12 @@
       <c r="BA1" s="9"/>
       <c r="BB1" s="9"/>
       <c r="BC1" s="9"/>
-    </row>
-    <row r="2" spans="1:55" x14ac:dyDescent="0.25">
+      <c r="BD1" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="BE1" s="12"/>
+    </row>
+    <row r="2" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1260,19 +1283,26 @@
       <c r="BC2" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="8" spans="1:55" x14ac:dyDescent="0.25">
+      <c r="BD2" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BE2" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="1:57" x14ac:dyDescent="0.25">
       <c r="BB8" s="5"/>
     </row>
-    <row r="14" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.25">
       <c r="G14" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="U1:AT1"/>
     <mergeCell ref="AV1:BC1"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:R1"/>
+    <mergeCell ref="BD1:BE1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>